<commit_message>
Budget template ships in three color themes (Emerald, Rose, Slate)
Theme-parameterize the budget build script and generate Rose and Slate
editions alongside Emerald — buyers get all three files in one purchase,
matching the multi-theme convention of bestselling templates. All three
recalculate clean with identical verified values. Listing gains a themes
bullet, the rose dashboard gallery shot, and an upload list of all
three files.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AkUe8kkZr9XS2EdNVryQd
</commit_message>
<xml_diff>
--- a/products/personal-budget-dashboard.xlsx
+++ b/products/personal-budget-dashboard.xlsx
@@ -1490,11 +1490,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="58128153"/>
-        <c:axId val="67598005"/>
+        <c:axId val="26204670"/>
+        <c:axId val="57299013"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="58128153"/>
+        <c:axId val="26204670"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1526,7 +1526,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67598005"/>
+        <c:crossAx val="57299013"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1534,7 +1534,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67598005"/>
+        <c:axId val="57299013"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1576,7 +1576,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58128153"/>
+        <c:crossAx val="26204670"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1827,11 +1827,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="18841806"/>
-        <c:axId val="16665554"/>
+        <c:axId val="44970787"/>
+        <c:axId val="73422122"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="18841806"/>
+        <c:axId val="44970787"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1863,7 +1863,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16665554"/>
+        <c:crossAx val="73422122"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1871,7 +1871,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16665554"/>
+        <c:axId val="73422122"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1913,7 +1913,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18841806"/>
+        <c:crossAx val="44970787"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7375,7 +7375,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22F1A067-91A9-4C28-AC5C-90FB24B27915}</x14:id>
+          <x14:id>{C896CE29-AA88-43B1-8A8E-DB9EEE85EBD7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -7398,7 +7398,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22F1A067-91A9-4C28-AC5C-90FB24B27915}">
+          <x14:cfRule type="dataBar" id="{C896CE29-AA88-43B1-8A8E-DB9EEE85EBD7}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -9661,7 +9661,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B05C78A4-CDCE-49FB-B346-DBD499943578}</x14:id>
+          <x14:id>{F1AB896F-C242-4540-9297-34D880A0DDF8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9677,7 +9677,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B05C78A4-CDCE-49FB-B346-DBD499943578}">
+          <x14:cfRule type="dataBar" id="{F1AB896F-C242-4540-9297-34D880A0DDF8}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>